<commit_message>
Ajout Recherche Machine (manque l'affichage par projet), calculs ORTEMS en Python,  Fix des problèmes de label, de mise à jour, etc., un peu de refactoring
</commit_message>
<xml_diff>
--- a/template/ortems_template.xlsx
+++ b/template/ortems_template.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adonfut\Desktop\Code\HET_3\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0FD7427-0ECA-473D-BF97-D0A6365B8C10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{955483CB-91A4-4F23-91B5-D7876E74F554}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="2415" windowWidth="21840" windowHeight="13140" xr2:uid="{3368FBE2-D29E-4C54-8DC2-E63CFA051357}"/>
   </bookViews>
   <sheets>
     <sheet name="prepa ORTEMS" sheetId="1" r:id="rId1"/>
-    <sheet name="Calculs" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
   <si>
     <t>HET tot</t>
   </si>
@@ -187,33 +186,6 @@
   </si>
   <si>
     <t>Système contrôle commande - électronique de puissance  Charge2</t>
-  </si>
-  <si>
-    <t>Nbr Projecteurs</t>
-  </si>
-  <si>
-    <t>Délair réel étude</t>
-  </si>
-  <si>
-    <t>Démarrage (mois)</t>
-  </si>
-  <si>
-    <t>Délai étude productif</t>
-  </si>
-  <si>
-    <t>Taux de productivité</t>
-  </si>
-  <si>
-    <t>Heures prises en compte</t>
-  </si>
-  <si>
-    <t>Délai brut (mois)</t>
-  </si>
-  <si>
-    <t>Congés (mois)</t>
-  </si>
-  <si>
-    <t>% Congés</t>
   </si>
 </sst>
 </file>
@@ -223,14 +195,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -247,7 +212,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -263,18 +228,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -303,11 +256,10 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -315,7 +267,7 @@
     <xf numFmtId="1" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
@@ -331,23 +283,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Pourcentage" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -791,10 +729,7 @@
         <f>SUM(C2:AX2)</f>
         <v>0</v>
       </c>
-      <c r="B2" s="3">
-        <f>Calculs!I3</f>
-        <v>0.5</v>
-      </c>
+      <c r="B2" s="3"/>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -853,84 +788,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{220A9472-B1C5-4CC6-AD39-864D8A83FC35}">
-  <dimension ref="A2:I3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="13.7109375" customWidth="1"/>
-    <col min="2" max="2" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="1:9" s="8" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A2" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="B2" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="D2" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="E2" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="F2" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="G2" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="H2" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="I2" s="11" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="12">
-        <f>'prepa ORTEMS'!O2</f>
-        <v>0</v>
-      </c>
-      <c r="B3" s="15">
-        <v>1.5</v>
-      </c>
-      <c r="C3" s="14">
-        <f>(A3/7.7)/(365.25/12 * 5/7)/B3</f>
-        <v>0</v>
-      </c>
-      <c r="D3" s="10">
-        <v>0.55000000000000004</v>
-      </c>
-      <c r="E3" s="14">
-        <f>C3/D3</f>
-        <v>0</v>
-      </c>
-      <c r="F3" s="16">
-        <f>2/12</f>
-        <v>0.16666666666666666</v>
-      </c>
-      <c r="G3" s="13">
-        <f>E3*F3</f>
-        <v>0</v>
-      </c>
-      <c r="H3" s="10">
-        <v>0.5</v>
-      </c>
-      <c r="I3" s="17">
-        <f>H3+E3+G3</f>
-        <v>0.5</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>